<commit_message>
Fix heading underlines, hero arrows, and mobile CTA padding.
Match accent bars to the content_four pattern, keep slider arrows off copy on smaller viewports, and restore honest QC sheet statuses.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/KES_feedback-to-dev-2026-09-29.xlsx
+++ b/docs/KES_feedback-to-dev-2026-09-29.xlsx
@@ -622,7 +622,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G48"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="5" customWidth="1" style="31" min="1" max="1"/>
     <col width="18" customWidth="1" style="31" min="2" max="2"/>
@@ -650,7 +650,7 @@
       </c>
       <c r="D1" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E1" s="13" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="D2" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E2" s="20" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="D4" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E4" s="20" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Waiting for</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E12" s="20" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E18" s="20" t="inlineStr">
@@ -1205,7 +1205,7 @@
       <c r="C19" s="25" t="n"/>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E19" s="13" t="n"/>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E20" s="20" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E26" s="20" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="D28" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E30" s="20" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E32" s="20" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E34" s="20" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="D36" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E36" s="20" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="D38" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E38" s="20" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="D40" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E40" s="20" t="inlineStr">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="D42" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E42" s="20" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="D44" s="19" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="E44" s="20" t="inlineStr">
@@ -3085,7 +3085,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="3" customWidth="1" style="31" min="1" max="1"/>
     <col width="30" customWidth="1" style="31" min="2" max="2"/>
@@ -3156,7 +3156,7 @@
         </is>
       </c>
       <c r="C7" s="11" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
@@ -3175,7 +3175,7 @@
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
@@ -3194,7 +3194,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
@@ -3213,7 +3213,7 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>

</xml_diff>